<commit_message>
V1.9.11. Ran DRC, added calculations for the antenna with ferrite.
</commit_message>
<xml_diff>
--- a/antenna calculations/cap_ind_calculations.xlsx
+++ b/antenna calculations/cap_ind_calculations.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveuclac-my.sharepoint.com/personal/rmaperu_ucl_ac_uk/Documents/Projects/sVNS_15_chan_circular_patch_antenna/sVNS_15chan_circular_antenna_board/antenna calculations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="11_F25DC773A252ABDACC104826899D6C0E5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E61CC906-286A-4C85-8950-415587E5AF44}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="11_F25DC773A252ABDACC104826899D6C0E5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD000344-3B93-4AE2-BE61-D762514B0F3D}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="1704" windowWidth="21600" windowHeight="11232" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calc_pcb_30mm" sheetId="5" r:id="rId1"/>
     <sheet name="real_pcb_30mm" sheetId="6" r:id="rId2"/>
-    <sheet name="calc_pcb_40mm" sheetId="1" r:id="rId3"/>
-    <sheet name="calc_pcb_35mm" sheetId="2" r:id="rId4"/>
-    <sheet name="real_pcb_40mm" sheetId="3" r:id="rId5"/>
-    <sheet name="real_pcb_35mm" sheetId="4" r:id="rId6"/>
+    <sheet name="real_pcb_30mm_ferrite" sheetId="7" r:id="rId3"/>
+    <sheet name="calc_pcb_40mm" sheetId="1" r:id="rId4"/>
+    <sheet name="calc_pcb_35mm" sheetId="2" r:id="rId5"/>
+    <sheet name="real_pcb_40mm" sheetId="3" r:id="rId6"/>
+    <sheet name="real_pcb_35mm" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
   <si>
     <t>C = 1/(4pi^2 f^2 L)</t>
   </si>
@@ -57,6 +59,48 @@
   </si>
   <si>
     <t>Ctune</t>
+  </si>
+  <si>
+    <t>Antenna no</t>
+  </si>
+  <si>
+    <t>L (no ferrite) uH</t>
+  </si>
+  <si>
+    <t>L (with ferrite) uH</t>
+  </si>
+  <si>
+    <t>Q (no ferrite) -</t>
+  </si>
+  <si>
+    <t>Q (with ferrite) -</t>
+  </si>
+  <si>
+    <t>Antenna no 1 - tuned to 13.56 MHz + 50 pF</t>
+  </si>
+  <si>
+    <t>Res freq (no ferrite) MHz</t>
+  </si>
+  <si>
+    <t>Res freq (with ferrite) MHz</t>
+  </si>
+  <si>
+    <t>Res freq (no ferrite) MHz + 50 pF</t>
+  </si>
+  <si>
+    <t>Res freq (with ferrite) MHz + 50 pF</t>
+  </si>
+  <si>
+    <t>&gt;20</t>
+  </si>
+  <si>
+    <t>Cap for res no ferrite (predicted) (pF)</t>
+  </si>
+  <si>
+    <t>Cap for res w/ ferrite (predicted) (pF)</t>
+  </si>
+  <si>
+    <t>Fres (w/ ferrite) MHz (+47 pF) || 12.5 pF</t>
   </si>
 </sst>
 </file>
@@ -92,10 +136,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,6 +535,147 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE657007-3958-488F-AF69-3897DEC76843}">
+  <dimension ref="B2:K9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="22.5546875" customWidth="1"/>
+    <col min="9" max="9" width="21.21875" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" customWidth="1"/>
+    <col min="11" max="11" width="22.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1.65917</v>
+      </c>
+      <c r="D4">
+        <v>2.28539</v>
+      </c>
+      <c r="E4">
+        <v>87.228999999999999</v>
+      </c>
+      <c r="F4">
+        <v>83.490399999999994</v>
+      </c>
+      <c r="H4" s="2">
+        <f>10^12*1/(4*PI()^2*13560000^2*C4*10^-6)</f>
+        <v>83.029036402618289</v>
+      </c>
+      <c r="I4" s="2">
+        <f>10^12*1/(4*PI()^2*13560000^2*D4*10^-6)</f>
+        <v>60.27823974382148</v>
+      </c>
+      <c r="K4">
+        <v>13.798999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.6599600000000001</v>
+      </c>
+      <c r="D5">
+        <v>2.2848899999999999</v>
+      </c>
+      <c r="E5">
+        <v>87.718900000000005</v>
+      </c>
+      <c r="F5">
+        <v>85.266499999999994</v>
+      </c>
+      <c r="H5" s="2">
+        <f>10^12*1/(4*PI()^2*13560000^2*C5*10^-6)</f>
+        <v>82.989521631926166</v>
+      </c>
+      <c r="I5" s="2">
+        <f>10^12*1/(4*PI()^2*13560000^2*D5*10^-6)</f>
+        <v>60.291430365633438</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+    </row>
+    <row r="8" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="2">
+        <v>3.5211399999999999</v>
+      </c>
+      <c r="F9">
+        <v>42.750599999999999</v>
+      </c>
+      <c r="G9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9">
+        <v>19.311</v>
+      </c>
+      <c r="I9">
+        <v>14.3918</v>
+      </c>
+      <c r="J9">
+        <v>12.8666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -550,7 +738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC1D79CD-43B2-46E8-A72D-23F6BD10A5C0}">
   <dimension ref="B2:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -602,7 +790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D5C186B-44B9-41D8-A12A-BBC77CF93496}">
   <dimension ref="B2:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -657,7 +845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07B55C1-00B9-4381-A350-547C8B65022E}">
   <dimension ref="B2:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>